<commit_message>
Add job scraper results - 2026-06-24
</commit_message>
<xml_diff>
--- a/results/cybersecurity-jobs-2026-06-24.xlsx
+++ b/results/cybersecurity-jobs-2026-06-24.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J138"/>
+  <dimension ref="A1:J120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -881,17 +881,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>IAM Engineer Sr - Separation of Duties</t>
+          <t>Senior Ping Identity Engineer</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Huntington National Bank</t>
+          <t>The Select Group</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Minnetonka, MN</t>
+          <t>San Diego, CA</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
@@ -900,7 +900,7 @@
       <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -917,26 +917,22 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Senior IAM Engineer – Identity Governance &amp; Administration</t>
+          <t>Ping Identity Engineer</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Moderna</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Cambridge, MA</t>
-        </is>
-      </c>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -953,17 +949,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Senior Ping Identity Engineer</t>
+          <t>IAM Solutions Engineer</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>The Select Group</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>San Diego, CA</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr"/>
@@ -972,7 +968,7 @@
       <c r="G13" s="4" t="inlineStr"/>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -989,26 +985,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Identity &amp; Automation Engineer</t>
+          <t>SailPoint IIQ Architect (IAM)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Sonatus</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Sunnyvale, CA</t>
-        </is>
-      </c>
+          <t>Connect Tech+Talent</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1025,12 +1017,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Ping Identity Engineer</t>
+          <t>Senior Security Engineer</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Jobgether</t>
+          <t>ARK Solutions, Inc.</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
@@ -1040,7 +1032,7 @@
       <c r="G15" s="4" t="inlineStr"/>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1057,28 +1049,20 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Identity and Access Management Engineer</t>
+          <t>IAM Security Engineer</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ECS</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Fairfax, VA</t>
-        </is>
-      </c>
+          <t>Chasepro</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+      <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -1093,28 +1077,20 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>IAM Solutions Engineer</t>
+          <t>IAM Security Engineer</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Alignerr</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Seattle, WA</t>
-        </is>
-      </c>
+          <t>NLB Services</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="H17" s="4" t="inlineStr"/>
       <c r="I17" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -1129,28 +1105,20 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Lead Engineer, Identity Management</t>
+          <t>IAM Security Engineer</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Sony Pictures Entertainment</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Culver City, CA</t>
-        </is>
-      </c>
+          <t>Axis Technologies</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -1165,28 +1133,24 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Systems Engineer II - PAM</t>
+          <t>IAM Security Engineer - W2 Only</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Early Warning</t>
+          <t>HonorVet Technologies</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Chicago, IL</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr"/>
       <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -1201,28 +1165,24 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Senior Identity and Access Management (IAM) Engineer</t>
+          <t>Security Analyst / Engineer (IAM &amp; Splunk)</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>1X</t>
+          <t>The Fountain Group</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>San Carlos, CA</t>
+          <t>North Carolina, United States</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+      <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -1237,12 +1197,12 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>IAM Security Engineer</t>
+          <t>Security Engineer</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Chasepro</t>
+          <t>Soho Square Solutions</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
@@ -1265,12 +1225,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>IAM Security Engineer</t>
+          <t>Cloud Security Analyst</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>NLB Services</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr"/>
@@ -1293,23 +1253,43 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>IAM Security Engineer</t>
+          <t>IAM Architect</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Axis Technologies</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr"/>
+          <t>Tata Consultancy Services (TCS)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Alpharetta, GA, US</t>
+        </is>
+      </c>
       <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>120000.0</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>130000.0</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1321,27 +1301,43 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>IAM Security Engineer - W2 Only</t>
+          <t>Identity Provider Manager (IdP) Project Manager</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HonorVet Technologies</t>
+          <t>General Dynamics Information Technology</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>Fort Meade, MD, US</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>148750.0</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>201250.0</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
@@ -1353,27 +1349,47 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Security Analyst / Engineer (IAM &amp; Splunk)</t>
+          <t>Sr Systems Security Engineer / Sr. Core Applications Administrator</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>The Fountain Group</t>
+          <t>Sierra Nevada Corporation</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>North Carolina, United States</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Lone Tree, CO, US</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>143487.0</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>197294.0</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -1385,23 +1401,43 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>IAM Security Engineer (W2)</t>
+          <t>IAM Engineer</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>PTR Global</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
+          <t>Accenture Federal Services</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Washington, DC, US</t>
+        </is>
+      </c>
       <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>64000.0</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>221100.0</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
@@ -1413,23 +1449,43 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Security Engineer</t>
+          <t>CyberArk PAM Operations Engineer</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Soho Square Solutions</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
+          <t>Accenture Federal Services</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Washington, DC, US</t>
+        </is>
+      </c>
       <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>64000.0</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>124200.0</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -1441,27 +1497,31 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Senior Identity Management Engineer</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Aurora</t>
-        </is>
-      </c>
+          <t>Cybersecurity Engineer</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>San Francisco, CA</t>
+          <t>Arlington, VA, US</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -1473,38 +1533,30 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>IAM Architect</t>
+          <t>Information Security Manager, IAM</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Tata Consultancy Services (TCS)</t>
+          <t>At Home The Home Decor Superstore</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Alpharetta, GA, US</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>120000.0</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>130000.0</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Coppell, TX, US</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -1521,28 +1573,32 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Identity Provider Manager (IdP) Project Manager</t>
+          <t>Cybersecurity SRE Principal Engineer</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>General Dynamics Information Technology</t>
+          <t>Wells Fargo</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Fort Meade, MD, US</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
+          <t>Columbus, OH, US</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>148750.0</t>
+          <t>159000.0</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>201250.0</t>
+          <t>254000.0</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1552,7 +1608,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -1569,17 +1625,17 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Sr Systems Security Engineer / Sr. Core Applications Administrator</t>
+          <t>ZERO TRUST (ZT) IDENTITY &amp; CREDENTIAL MANAGEMENT SME</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Sierra Nevada Corporation</t>
+          <t>J.B. Hunt</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Lone Tree, CO, US</t>
+          <t>Arlington, VA, US</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1587,24 +1643,12 @@
           <t>fulltime</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>143487.0</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>197294.0</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr"/>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
@@ -1621,28 +1665,28 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>IAM Engineer</t>
+          <t>Privileged Access Management - Conjur Operations Engineer</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Accenture Federal Services</t>
+          <t>Nomura</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC, US</t>
+          <t>Jacksonville, FL, US</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>64000.0</t>
+          <t>95000.0</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>221100.0</t>
+          <t>110000.0</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1652,7 +1696,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -1669,38 +1713,22 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>CyberArk PAM Operations Engineer</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Accenture Federal Services</t>
-        </is>
-      </c>
+          <t>Identity and Access Management Consultant</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr"/>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Washington, DC, US</t>
+          <t>Atlanta, GA, US</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>64000.0</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>124200.0</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr"/>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I33" s="4" t="inlineStr">
@@ -1717,23 +1745,19 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer</t>
+          <t>Identity and Access Management Leader</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Arlington, VA, US</t>
+          <t>Atlanta, GA, US</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="G34" s="2" t="inlineStr"/>
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>2026-06-22</t>
@@ -1753,17 +1777,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Information Security Manager, IAM</t>
+          <t>Security Engineer</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>At Home The Home Decor Superstore</t>
+          <t>Integris</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Coppell, TX, US</t>
+          <t>Remote, US</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1776,7 +1800,7 @@
       <c r="G35" s="4" t="inlineStr"/>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -1793,47 +1817,31 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity SRE Principal Engineer</t>
+          <t>Systems Engineer II - PAM</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Wells Fargo</t>
+          <t>Early Warning</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Columbus, OH, US</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>159000.0</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>254000.0</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Scottsdale, AZ</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
@@ -1845,35 +1853,27 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>ZERO TRUST (ZT) IDENTITY &amp; CREDENTIAL MANAGEMENT SME</t>
+          <t>PAM Engineer</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>J.B. Hunt</t>
+          <t>Programmers.io</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Arlington, VA, US</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
+      <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -1885,28 +1885,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Privileged Access Management - Conjur Operations Engineer</t>
+          <t>IAM Cloud Governance Engineer</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Nomura</t>
+          <t>KeyBank</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Jacksonville, FL, US</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
+          <t>Brooklyn, OH, US</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>95000.0</t>
+          <t>80000.0</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>110000.0</t>
+          <t>150000.0</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -1933,16 +1937,24 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Identity and Access Management Consultant</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr"/>
+          <t>IAM Engineer Sr - Separation of Duties</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Huntington Bank</t>
+        </is>
+      </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Atlanta, GA, US</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr"/>
+          <t>Minnetonka, MN, US</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="4" t="inlineStr"/>
@@ -1965,22 +1977,26 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Identity and Access Management Leader</t>
+          <t>Corporate Security Architect</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Atlanta, GA, US</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr"/>
+          <t>Los Angeles, CA, US</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -1997,17 +2013,17 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Security Engineer</t>
+          <t>Cybersecurity Engineer</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Integris</t>
+          <t>Dutch Bros Coffee</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Remote, US</t>
+          <t>Tempe, AZ, US</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2020,7 +2036,7 @@
       <c r="G41" s="4" t="inlineStr"/>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
@@ -2037,27 +2053,35 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>PAM Engineer</t>
+          <t>Sr Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Northwest Partners</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
+          <t>Blue Cross Blue Shield of Nebraska</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Omaha, NE, US</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -2069,23 +2093,47 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>PAM Beyond Trust Password Safe SME</t>
+          <t>Senior CyberArk Engineer</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>PineQ Lab Technology</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr"/>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-      <c r="H43" s="4" t="inlineStr"/>
+          <t>SAIC</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Washington, DC, US</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>120001.0</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>160000.0</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
@@ -2097,32 +2145,28 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>IAM Cloud Governance Engineer</t>
+          <t>Cyber Managed Services - SDC IAM - Senior</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>KeyBank</t>
+          <t>EY</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Brooklyn, OH, US</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Dallas, TX, US</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>80000.0</t>
+          <t>77500.0</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>150000.0</t>
+          <t>160500.0</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2132,7 +2176,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2149,22 +2193,22 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>IAM Engineer Sr - Separation of Duties</t>
+          <t>Ping Identity Engineer</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Huntington Bank</t>
+          <t>Airitos</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Minnetonka, MN, US</t>
+          <t>Remote, US</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>fulltime</t>
+          <t>contract</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr"/>
@@ -2172,7 +2216,7 @@
       <c r="G45" s="4" t="inlineStr"/>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
@@ -2189,13 +2233,17 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Corporate Security Architect</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
+          <t>Identity &amp; Access Management (IAM) Engineer</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Customers Bank</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Los Angeles, CA, US</t>
+          <t>Malvern, PA, US</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2208,7 +2256,7 @@
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2225,17 +2273,17 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer</t>
+          <t>PKI Security Analyst</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Dutch Bros Coffee</t>
+          <t>MetLife</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Tempe, AZ, US</t>
+          <t>Cary, NC, US</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2243,12 +2291,24 @@
           <t>fulltime</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>70000.0</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>90000.0</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
@@ -2265,17 +2325,17 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Sr Cloud Security Engineer</t>
+          <t>Lead, Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Blue Cross Blue Shield of Nebraska</t>
+          <t>W.W. Williams Company</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Omaha, NE, US</t>
+          <t>Irving, TX, US</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2288,7 +2348,7 @@
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2305,42 +2365,22 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Senior CyberArk Engineer</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
+          <t>IAM Engineer</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr"/>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Washington, DC, US</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>120001.0</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>160000.0</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Austin, TX, US</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
       <c r="H49" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="I49" s="4" t="inlineStr">
@@ -2357,43 +2397,27 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Cyber Managed Services - SDC IAM - Senior</t>
+          <t>Identity &amp; Access Management (IAM) Analyst</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>EY</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Dallas, TX, US</t>
-        </is>
-      </c>
+          <t>Alignerr</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
       <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>77500.0</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>160500.0</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J50" s="3" t="inlineStr">
@@ -2405,35 +2429,27 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Ping Identity Engineer</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Airitos</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>Remote, US</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>contract</t>
-        </is>
-      </c>
+          <t>InterEx Group</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr"/>
+      <c r="D51" s="4" t="inlineStr"/>
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr"/>
       <c r="G51" s="4" t="inlineStr"/>
       <c r="H51" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
@@ -2445,35 +2461,31 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Identity &amp; Access Management (IAM) Engineer</t>
+          <t>Senior Technology Security Engineer (IAM)</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Customers Bank</t>
+          <t>Pointwest-North America</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Malvern, PA, US</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Des Moines, IA</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr"/>
       <c r="E52" s="2" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J52" s="3" t="inlineStr">
@@ -2485,47 +2497,31 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>PKI Security Analyst</t>
+          <t>Identity &amp; Access Management Engineer (Hybrid/Remote)</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>MetLife</t>
+          <t>MKS Inc.</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Cary, NC, US</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>70000.0</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>90000.0</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Rochester, NY</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr"/>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J53" s="5" t="inlineStr">
@@ -2537,35 +2533,27 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Lead, Cyber Security Engineer</t>
+          <t>Cybersecurity Engineer (TS Cleared)</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>W.W. Williams Company</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Irving, TX, US</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Kentro</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr"/>
       <c r="E54" s="2" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J54" s="3" t="inlineStr">
@@ -2577,13 +2565,17 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>IAM Engineer</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr"/>
+          <t>IAM Practitioner</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Computershare U.S.</t>
+        </is>
+      </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Austin, TX, US</t>
+          <t>Canton, MA</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr"/>
@@ -2592,12 +2584,12 @@
       <c r="G55" s="4" t="inlineStr"/>
       <c r="H55" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -2609,12 +2601,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Identity &amp; Access Management (IAM) Analyst</t>
+          <t>IAM Analyst</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Alignerr</t>
+          <t>Insight Global</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr"/>
@@ -2624,7 +2616,7 @@
       <c r="G56" s="2" t="inlineStr"/>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -2646,17 +2638,21 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>InterEx Group</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr"/>
+          <t>Russell Tobin</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>California, United States</t>
+        </is>
+      </c>
       <c r="D57" s="4" t="inlineStr"/>
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr"/>
       <c r="G57" s="4" t="inlineStr"/>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I57" s="4" t="inlineStr">
@@ -2673,12 +2669,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer (TS Cleared)</t>
+          <t>Penetration Tester - Contract</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Kentro</t>
+          <t>Bishop Fox</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr"/>
@@ -2688,7 +2684,7 @@
       <c r="G58" s="2" t="inlineStr"/>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -2705,22 +2701,26 @@
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>IAM Analyst</t>
+          <t>Cyber Security Engineer (100% Remote)</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Insight Global</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr"/>
+          <t>Motion Recruitment</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
       <c r="D59" s="4" t="inlineStr"/>
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr"/>
       <c r="G59" s="4" t="inlineStr"/>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
@@ -2737,17 +2737,17 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security Analyst</t>
+          <t>Security Solutions Senior Consultant – CyberArk</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Russell Tobin</t>
+          <t>World Wide Technology</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>California, United States</t>
+          <t>New Home, MO</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -2756,7 +2756,7 @@
       <c r="G60" s="2" t="inlineStr"/>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -2773,17 +2773,17 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer (100% Remote)</t>
+          <t>Senior Cybersecurity Operations Engineer (FedRAMP Readiness)</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Motion Recruitment</t>
+          <t>Revel IT</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Columbus, Ohio Metropolitan Area</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr"/>
@@ -2792,7 +2792,7 @@
       <c r="G61" s="4" t="inlineStr"/>
       <c r="H61" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
@@ -2809,19 +2809,15 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Senior Cybersecurity Operations Engineer (FedRAMP Readiness)</t>
+          <t>Security Engineer - Email Security Application</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Revel IT</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Columbus, Ohio Metropolitan Area</t>
-        </is>
-      </c>
+          <t>VAILEXA</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr"/>
       <c r="D62" s="2" t="inlineStr"/>
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr"/>
@@ -2845,24 +2841,24 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Security Engineer - Email Security Application</t>
+          <t>Cyber Security Engineer - 17174</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>VAILEXA</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr"/>
+          <t>Seneca Resources Company, LLC</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Virginia, United States</t>
+        </is>
+      </c>
       <c r="D63" s="4" t="inlineStr"/>
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr"/>
       <c r="G63" s="4" t="inlineStr"/>
-      <c r="H63" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+      <c r="H63" s="4" t="inlineStr"/>
       <c r="I63" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -2877,19 +2873,15 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer - 17174</t>
+          <t>Sr. Cybersecurity Engineer</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Seneca Resources Company, LLC</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Virginia, United States</t>
-        </is>
-      </c>
+          <t>Hays</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr"/>
       <c r="D64" s="2" t="inlineStr"/>
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
@@ -2909,15 +2901,19 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Sr. Cybersecurity Engineer</t>
+          <t>Lead CyberSecurity Analyst</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Hays</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr"/>
+          <t>Prestige Staffing</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
       <c r="D65" s="4" t="inlineStr"/>
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr"/>
@@ -2937,15 +2933,19 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security Analyst</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>S Piper Staffing LLC</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr"/>
+          <t>Seneca Resources</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Virginia, United States</t>
+        </is>
+      </c>
       <c r="D66" s="2" t="inlineStr"/>
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
@@ -2965,15 +2965,19 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Splunk Security Engineer</t>
+          <t>Remote | Cybersecurity AI Safety Engineer — $50–$80/hour</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>NLB Services</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr"/>
+          <t>24-MAG</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
       <c r="D67" s="4" t="inlineStr"/>
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr"/>
@@ -2993,15 +2997,19 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Product Security Engineer</t>
+          <t>Privileged Access Manager Engineer</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Cypress HCM</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr"/>
+          <t>Booz Allen Hamilton</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Arlington, VA</t>
+        </is>
+      </c>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
@@ -3021,17 +3029,17 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Lead CyberSecurity Analyst</t>
+          <t>Cyber Security Engineer</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Prestige Staffing</t>
+          <t>NLB Services</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr"/>
@@ -3053,17 +3061,17 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer</t>
+          <t>Senior Security Engineer</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Seneca Resources</t>
+          <t>ANDREW an Amphenol company</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Virginia, United States</t>
+          <t>Richardson, TX</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
@@ -3085,23 +3093,47 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Security Engineer</t>
+          <t>Cybersecurity Engineer</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>GAC Solutions</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr"/>
-      <c r="D71" s="4" t="inlineStr"/>
-      <c r="E71" s="4" t="inlineStr"/>
-      <c r="F71" s="4" t="inlineStr"/>
-      <c r="G71" s="4" t="inlineStr"/>
-      <c r="H71" s="4" t="inlineStr"/>
+          <t>Apollo Information Systems</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>80000.0</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>120000.0</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J71" s="5" t="inlineStr">
@@ -3113,23 +3145,47 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Recruiter</t>
+          <t>Cybersecurity Advisor II</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Bernard Nickels &amp; Associates</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr"/>
-      <c r="D72" s="2" t="inlineStr"/>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
+          <t>Apollo Information Systems</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>120000.0</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>160000.0</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
@@ -3141,17 +3197,17 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer</t>
+          <t>Security Engineer, Application Security</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Apollo Information Systems</t>
+          <t>SERVAL</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>San Francisco, CA, US</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -3161,12 +3217,12 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>80000.0</t>
+          <t>200000.0</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>120000.0</t>
+          <t>325000.0</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr">
@@ -3193,39 +3249,23 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Advisor II</t>
+          <t>Application Security Analyst</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Apollo Information Systems</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>120000.0</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>160000.0</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
       <c r="H74" s="2" t="inlineStr">
         <is>
           <t>2026-06-23</t>
@@ -3233,7 +3273,7 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
@@ -3245,47 +3285,31 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>Security Engineer, Application Security</t>
+          <t>Sr Endpoint Security Engineer</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>SERVAL</t>
+          <t>Stefanini North America and APAC</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>San Francisco, CA, US</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>200000.0</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>325000.0</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>New York, United States</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J75" s="5" t="inlineStr">
@@ -3297,22 +3321,26 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Application Security Analyst</t>
+          <t>Data Security Engineer</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Alignerr</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr"/>
+          <t>Medal</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
       <c r="D76" s="2" t="inlineStr"/>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr"/>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -3329,22 +3357,26 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>Cloud Security Engineer</t>
+          <t>Sr Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>MoonPay</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr"/>
+          <t>BJ's Wholesale Club</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Marlborough, MA</t>
+        </is>
+      </c>
       <c r="D77" s="4" t="inlineStr"/>
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr"/>
       <c r="G77" s="4" t="inlineStr"/>
       <c r="H77" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
@@ -3361,17 +3393,17 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Cloud Security Engineer, Sr</t>
+          <t>Sr Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Old National Bank</t>
+          <t>Blue Cross and Blue Shield of Nebraska</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Evansville, IN</t>
+          <t>Omaha, NE</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr"/>
@@ -3380,7 +3412,7 @@
       <c r="G78" s="2" t="inlineStr"/>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3397,17 +3429,17 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>Cyber Security Engineer (Cloud Security)</t>
+          <t>Platform Security Engineer 2</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Garmin</t>
+          <t>HDR</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>Olathe, KS</t>
+          <t>Portland, OR</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr"/>
@@ -3433,26 +3465,22 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Security Engineer</t>
+          <t>Senior Security Engineer</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Sonata Software North America Inc.</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>Irving, TX</t>
-        </is>
-      </c>
+          <t>Covenant HR</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr"/>
       <c r="D80" s="2" t="inlineStr"/>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -3469,22 +3497,26 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>Sr Security Engineer — Specialist (IAM / Data Protection / Forensics)</t>
+          <t>Security Engineer, Infrastructure Security</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Envision Technology Solutions</t>
-        </is>
-      </c>
-      <c r="C81" s="4" t="inlineStr"/>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
       <c r="D81" s="4" t="inlineStr"/>
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr"/>
       <c r="G81" s="4" t="inlineStr"/>
       <c r="H81" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I81" s="4" t="inlineStr">
@@ -3501,17 +3533,17 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Infrastructure Security Engineer</t>
+          <t>Staff Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Opendoor</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Seattle, WA</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr"/>
@@ -3520,7 +3552,7 @@
       <c r="G82" s="2" t="inlineStr"/>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -3537,28 +3569,20 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>IT Security Engineer Senior</t>
+          <t>Security Engineer</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Texas Roadhouse</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>Louisville, KY</t>
-        </is>
-      </c>
+          <t>Blue Bridge People</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr"/>
       <c r="D83" s="4" t="inlineStr"/>
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr"/>
       <c r="G83" s="4" t="inlineStr"/>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="H83" s="4" t="inlineStr"/>
       <c r="I83" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -3573,28 +3597,20 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Security Engineer - Identity Services Engine</t>
+          <t>Security Engineer</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>VAILEXA</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Seattle, WA</t>
-        </is>
-      </c>
+          <t>Net2Source (N2S)</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr"/>
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr"/>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+      <c r="H84" s="2" t="inlineStr"/>
       <c r="I84" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -3609,19 +3625,15 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>Cloud Security Engineer</t>
+          <t>Splunk Security Engineer</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Thales</t>
-        </is>
-      </c>
-      <c r="C85" s="4" t="inlineStr">
-        <is>
-          <t>Austin, TX</t>
-        </is>
-      </c>
+          <t>NLB Services</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr"/>
       <c r="D85" s="4" t="inlineStr"/>
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr"/>
@@ -3641,19 +3653,15 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Platform Security Engineer</t>
+          <t>Senior Security Engineer</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Superhuman</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>Seattle, WA</t>
-        </is>
-      </c>
+          <t>Insight Global</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr"/>
       <c r="D86" s="2" t="inlineStr"/>
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
@@ -3673,17 +3681,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>Cloud Security Engineer (AWS)</t>
+          <t>Senior Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Pedestal Health</t>
+          <t>Vanguard</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Durham, NC</t>
+          <t>Charlotte, NC</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr"/>
@@ -3705,15 +3713,19 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Senior Security Engineer</t>
+          <t>Cloud Security Engineer</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Insight Global</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr"/>
+          <t>Bates White Economic Consulting</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Washington, DC</t>
+        </is>
+      </c>
       <c r="D88" s="2" t="inlineStr"/>
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
@@ -3733,27 +3745,43 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>Remote | Cybersecurity AI Safety Engineer — $50–$80/hour</t>
+          <t>Senior Advisor, Incident Response</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>24-MAG</t>
+          <t>Sophos Technology GmbH</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>Dallas, TX, US</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr"/>
-      <c r="E89" s="4" t="inlineStr"/>
-      <c r="F89" s="4" t="inlineStr"/>
-      <c r="G89" s="4" t="inlineStr"/>
-      <c r="H89" s="4" t="inlineStr"/>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>150000.0</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>250000.0</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J89" s="5" t="inlineStr">
@@ -3765,23 +3793,39 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Offensive Security Engineer</t>
+          <t>Senior Information Security Consultant (QSA)</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Covenant HR</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr"/>
-      <c r="D90" s="2" t="inlineStr"/>
+          <t>Sikich</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
@@ -3793,23 +3837,39 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Information Security Engineer (Level IV)</t>
+          <t>Principal Security Consultant - F5 Services</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>CBTS</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="inlineStr"/>
-      <c r="D91" s="4" t="inlineStr"/>
+          <t>World Wide Technology</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Remote, US</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr"/>
-      <c r="G91" s="4" t="inlineStr"/>
-      <c r="H91" s="4" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J91" s="5" t="inlineStr">
@@ -3821,28 +3881,32 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Senior Advisor, Incident Response</t>
+          <t>Information Security Consultant</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Sophos Technology GmbH</t>
+          <t>MassMutual</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Dallas, TX, US</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr"/>
+          <t>Springfield, MA, US</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>150000.0</t>
+          <t>86200.0</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>250000.0</t>
+          <t>113100.0</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -3869,17 +3933,17 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>Senior Information Security Consultant (QSA)</t>
+          <t>Principal Incident Response Security Consultant, Mandiant, Google Cloud</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Sikich</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Cambridge, MA, US</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -3887,8 +3951,16 @@
           <t>fulltime</t>
         </is>
       </c>
-      <c r="E93" s="4" t="inlineStr"/>
-      <c r="F93" s="4" t="inlineStr"/>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>168000.0</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>244000.0</t>
+        </is>
+      </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
           <t>USD</t>
@@ -3913,31 +3985,19 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Principal Security Consultant - F5 Services</t>
+          <t>Cybersecurity Defense Expert</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>World Wide Technology</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>Remote, US</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
+          <t>Alignerr</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="2" t="inlineStr"/>
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+      <c r="G94" s="2" t="inlineStr"/>
       <c r="H94" s="2" t="inlineStr">
         <is>
           <t>2026-06-23</t>
@@ -3945,7 +4005,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J94" s="3" t="inlineStr">
@@ -3957,47 +4017,31 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>Information Security Consultant</t>
+          <t>Cloud Security Senior Consultant - M365</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>MassMutual</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>Springfield, MA, US</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>86200.0</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>113100.0</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Kansas City, MO</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr"/>
+      <c r="E95" s="4" t="inlineStr"/>
+      <c r="F95" s="4" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr"/>
       <c r="H95" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J95" s="5" t="inlineStr">
@@ -4009,47 +4053,31 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Principal Incident Response Security Consultant, Mandiant, Google Cloud</t>
+          <t>Lead Penetration Tester</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Cambridge, MA, US</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>168000.0</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>244000.0</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>indeed</t>
+          <t>linkedin</t>
         </is>
       </c>
       <c r="J96" s="3" t="inlineStr">
@@ -4061,22 +4089,26 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>REMOTE Cybersecurity Governance Program Manager (ISP/ Telecom industry experience)</t>
+          <t>Cybersecurity Advisory Consultant</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Insight Global</t>
-        </is>
-      </c>
-      <c r="C97" s="4" t="inlineStr"/>
+          <t>Plante Moran</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Southfield, MI</t>
+        </is>
+      </c>
       <c r="D97" s="4" t="inlineStr"/>
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr"/>
       <c r="G97" s="4" t="inlineStr"/>
       <c r="H97" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I97" s="4" t="inlineStr">
@@ -4093,28 +4125,24 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>IT &amp; Cyber Security Consultant</t>
+          <t>Application Security Consultant, Mandiant, Google Cloud</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>OnTrac</t>
+          <t>Google</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Connecticut, United States</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr"/>
       <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
+      <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4129,28 +4157,24 @@
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer</t>
+          <t>Cyber Security Consultant</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Smithfield Foods</t>
+          <t>Idexcel</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>Suffolk, VA</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr"/>
       <c r="E99" s="4" t="inlineStr"/>
       <c r="F99" s="4" t="inlineStr"/>
       <c r="G99" s="4" t="inlineStr"/>
-      <c r="H99" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+      <c r="H99" s="4" t="inlineStr"/>
       <c r="I99" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4165,28 +4189,20 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>IT Incident Response and Forensics Consultant III</t>
+          <t>Penetration Tester</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Kaiser Permanente</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>Greensboro, NC</t>
-        </is>
-      </c>
+          <t>Akkodis</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr"/>
       <c r="D100" s="2" t="inlineStr"/>
       <c r="E100" s="2" t="inlineStr"/>
       <c r="F100" s="2" t="inlineStr"/>
       <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
+      <c r="H100" s="2" t="inlineStr"/>
       <c r="I100" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4201,28 +4217,24 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>Senior Cybersecurity Consultant (Vulnerability &amp; Threat Response)</t>
+          <t>Project Manager- Cybersecurity</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Motion Recruitment</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New Brunswick, NJ</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr"/>
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="4" t="inlineStr"/>
       <c r="G101" s="4" t="inlineStr"/>
-      <c r="H101" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
+      <c r="H101" s="4" t="inlineStr"/>
       <c r="I101" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4237,17 +4249,17 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Cyber Security Consultant</t>
+          <t>Principal Cloud Security Architect</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>ConfigUSA</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Burlington, MA</t>
+          <t>Austin, CO</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
@@ -4273,26 +4285,22 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>Cybersecurity Advisory Consultant</t>
+          <t>AI Security Architect</t>
         </is>
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Plante Moran</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>Southfield, MI</t>
-        </is>
-      </c>
+          <t>KPG99 INC</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr"/>
       <c r="D103" s="4" t="inlineStr"/>
       <c r="E103" s="4" t="inlineStr"/>
       <c r="F103" s="4" t="inlineStr"/>
       <c r="G103" s="4" t="inlineStr"/>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="I103" s="4" t="inlineStr">
@@ -4309,28 +4317,20 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Principal Cybersecurity Advisor (Cisco-Splunk) | Remote, USA</t>
+          <t>Information Security Principal Architect #11392</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Optiv</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>Leawood, KS</t>
-        </is>
-      </c>
+          <t>ECCO Select</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr"/>
       <c r="D104" s="2" t="inlineStr"/>
       <c r="E104" s="2" t="inlineStr"/>
       <c r="F104" s="2" t="inlineStr"/>
       <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
+      <c r="H104" s="2" t="inlineStr"/>
       <c r="I104" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4345,27 +4345,47 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>Cyber Security Consultant</t>
+          <t>IT Security Engineer II</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Idexcel</t>
+          <t>Endeavor Health</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>New York, NY</t>
-        </is>
-      </c>
-      <c r="D105" s="4" t="inlineStr"/>
-      <c r="E105" s="4" t="inlineStr"/>
-      <c r="F105" s="4" t="inlineStr"/>
-      <c r="G105" s="4" t="inlineStr"/>
-      <c r="H105" s="4" t="inlineStr"/>
+          <t>Arlington Heights, IL, US</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J105" s="5" t="inlineStr">
@@ -4377,20 +4397,28 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Consultant (Remote)</t>
+          <t>Incident Response Analyst</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr"/>
+          <t>Alignerr</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Dallas, TX</t>
+        </is>
+      </c>
       <c r="D106" s="2" t="inlineStr"/>
       <c r="E106" s="2" t="inlineStr"/>
       <c r="F106" s="2" t="inlineStr"/>
       <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4405,12 +4433,12 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>Cyber Security Risk Consultant (Remote)</t>
+          <t>Senior Application Security Engineer</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
+          <t>Insight Global</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr"/>
@@ -4418,7 +4446,11 @@
       <c r="E107" s="4" t="inlineStr"/>
       <c r="F107" s="4" t="inlineStr"/>
       <c r="G107" s="4" t="inlineStr"/>
-      <c r="H107" s="4" t="inlineStr"/>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4433,24 +4465,28 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity Advisor - Threat Management | Remote, MN, TX, TN, MO</t>
+          <t>Incident Response Lead, Cyber Security</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Optiv</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Houston, TX</t>
+          <t>Seattle, WA</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr"/>
-      <c r="H108" s="2" t="inlineStr"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4465,24 +4501,24 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>Cybersecurity Engineer</t>
+          <t>Security Engineer — Specialist (IAM / Data Protection / Forensics)</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Software Engineering Institute | Carnegie Mellon University</t>
-        </is>
-      </c>
-      <c r="C109" s="4" t="inlineStr">
-        <is>
-          <t>Pittsburgh, PA</t>
-        </is>
-      </c>
+          <t>SRM Digital LLC</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr"/>
       <c r="D109" s="4" t="inlineStr"/>
       <c r="E109" s="4" t="inlineStr"/>
       <c r="F109" s="4" t="inlineStr"/>
       <c r="G109" s="4" t="inlineStr"/>
-      <c r="H109" s="4" t="inlineStr"/>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
           <t>linkedin</t>
@@ -4497,19 +4533,15 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Senior Consultant, Cybersecurity | Forensic &amp; Litigation Consulting</t>
+          <t>Product Security Engineer</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>FTI Consulting</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>Washington, DC</t>
-        </is>
-      </c>
+          <t>Cypress HCM</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr"/>
       <c r="D110" s="2" t="inlineStr"/>
       <c r="E110" s="2" t="inlineStr"/>
       <c r="F110" s="2" t="inlineStr"/>
@@ -4529,27 +4561,43 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>Senior Associate Information Security Consultant</t>
+          <t>Penetration Tester - TS/SCI with Polygraph</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Truist</t>
+          <t>General Dynamics Information Technology</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>Charlotte, NC</t>
+          <t>McLean, VA, US</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr"/>
-      <c r="E111" s="4" t="inlineStr"/>
-      <c r="F111" s="4" t="inlineStr"/>
-      <c r="G111" s="4" t="inlineStr"/>
-      <c r="H111" s="4" t="inlineStr"/>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>152380.0</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr">
+        <is>
+          <t>206162.0</t>
+        </is>
+      </c>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J111" s="5" t="inlineStr">
@@ -4561,27 +4609,35 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Cyber Defense &amp; Engineering - Cloud Security Experienced Associate</t>
+          <t>Senior Penetration Tester</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>PwC</t>
+          <t>Quzara LLC</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Boston, MA</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr"/>
+          <t>Washington, DC, US</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>fulltime</t>
+        </is>
+      </c>
       <c r="E112" s="2" t="inlineStr"/>
       <c r="F112" s="2" t="inlineStr"/>
       <c r="G112" s="2" t="inlineStr"/>
-      <c r="H112" s="2" t="inlineStr"/>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J112" s="3" t="inlineStr">
@@ -4593,23 +4649,43 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>Security Consultant</t>
+          <t>Cyber Vulnerability Analyst - Penetration Tester - TS/SCI w/ Poly Required</t>
         </is>
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>Cyberr</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr"/>
+          <t>Parsons</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>Annapolis Junction, MD, US</t>
+        </is>
+      </c>
       <c r="D113" s="4" t="inlineStr"/>
-      <c r="E113" s="4" t="inlineStr"/>
-      <c r="F113" s="4" t="inlineStr"/>
-      <c r="G113" s="4" t="inlineStr"/>
-      <c r="H113" s="4" t="inlineStr"/>
+      <c r="E113" s="4" t="inlineStr">
+        <is>
+          <t>134100.0</t>
+        </is>
+      </c>
+      <c r="F113" s="4" t="inlineStr">
+        <is>
+          <t>241400.0</t>
+        </is>
+      </c>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>linkedin</t>
+          <t>indeed</t>
         </is>
       </c>
       <c r="J113" s="5" t="inlineStr">
@@ -4621,7 +4697,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Network &amp; Infrastructure Security Analyst</t>
+          <t>AI Security Penetration Tester</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -4629,11 +4705,7 @@
           <t>Alignerr</t>
         </is>
       </c>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>Boston, MA</t>
-        </is>
-      </c>
+      <c r="C114" s="2" t="inlineStr"/>
       <c r="D114" s="2" t="inlineStr"/>
       <c r="E114" s="2" t="inlineStr"/>
       <c r="F114" s="2" t="inlineStr"/>
@@ -4657,22 +4729,26 @@
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>Senior Information Security Engineer</t>
+          <t>Cybersecurity Penetration Testing Expert</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Prodware Solutions</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr"/>
+          <t>Alignerr</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
       <c r="D115" s="4" t="inlineStr"/>
       <c r="E115" s="4" t="inlineStr"/>
       <c r="F115" s="4" t="inlineStr"/>
       <c r="G115" s="4" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I115" s="4" t="inlineStr">
@@ -4689,12 +4765,12 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>AI Security Architect</t>
+          <t>AI Penetration Testing Expert</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>KPG99 INC</t>
+          <t>Alignerr</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr"/>
@@ -4704,7 +4780,7 @@
       <c r="G116" s="2" t="inlineStr"/>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr">
@@ -4721,7 +4797,7 @@
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>Principal Cloud Security Architect</t>
+          <t>Offensive Security Analyst (Structured / Non-Exploit)</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
@@ -4731,7 +4807,7 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>Austin, CO</t>
+          <t>Denver, CO</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr"/>
@@ -4740,7 +4816,7 @@
       <c r="G117" s="4" t="inlineStr"/>
       <c r="H117" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I117" s="4" t="inlineStr">
@@ -4757,22 +4833,26 @@
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Security Consultant</t>
+          <t>AI / Emerging Tech Security Analyst</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>CDW</t>
-        </is>
-      </c>
-      <c r="C118" s="2" t="inlineStr"/>
+          <t>Alignerr</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Boston, MA</t>
+        </is>
+      </c>
       <c r="D118" s="2" t="inlineStr"/>
       <c r="E118" s="2" t="inlineStr"/>
       <c r="F118" s="2" t="inlineStr"/>
       <c r="G118" s="2" t="inlineStr"/>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr">
@@ -4789,15 +4869,19 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>REMOTE: Security Architect (SAP)</t>
+          <t>Security Engineer - Identity Services Engine</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>IntePros</t>
-        </is>
-      </c>
-      <c r="C119" s="4" t="inlineStr"/>
+          <t>VAILEXA</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Seattle, WA</t>
+        </is>
+      </c>
       <c r="D119" s="4" t="inlineStr"/>
       <c r="E119" s="4" t="inlineStr"/>
       <c r="F119" s="4" t="inlineStr"/>
@@ -4821,12 +4905,12 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Enterprise Security Architect</t>
+          <t>Cyber Security Analyst</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Akkodis</t>
+          <t>S Piper Staffing LLC</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr"/>
@@ -4841,650 +4925,6 @@
         </is>
       </c>
       <c r="J120" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="4" t="inlineStr">
-        <is>
-          <t>Information Security Principal Architect #11392</t>
-        </is>
-      </c>
-      <c r="B121" s="4" t="inlineStr">
-        <is>
-          <t>ECCO Select</t>
-        </is>
-      </c>
-      <c r="C121" s="4" t="inlineStr"/>
-      <c r="D121" s="4" t="inlineStr"/>
-      <c r="E121" s="4" t="inlineStr"/>
-      <c r="F121" s="4" t="inlineStr"/>
-      <c r="G121" s="4" t="inlineStr"/>
-      <c r="H121" s="4" t="inlineStr"/>
-      <c r="I121" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J121" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>Cloud Security Analyst</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="inlineStr">
-        <is>
-          <t>Alignerr</t>
-        </is>
-      </c>
-      <c r="C122" s="2" t="inlineStr">
-        <is>
-          <t>Denver, CO</t>
-        </is>
-      </c>
-      <c r="D122" s="2" t="inlineStr"/>
-      <c r="E122" s="2" t="inlineStr"/>
-      <c r="F122" s="2" t="inlineStr"/>
-      <c r="G122" s="2" t="inlineStr"/>
-      <c r="H122" s="2" t="inlineStr"/>
-      <c r="I122" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J122" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="4" t="inlineStr">
-        <is>
-          <t>IT Security Engineer II</t>
-        </is>
-      </c>
-      <c r="B123" s="4" t="inlineStr">
-        <is>
-          <t>Endeavor Health</t>
-        </is>
-      </c>
-      <c r="C123" s="4" t="inlineStr">
-        <is>
-          <t>Arlington Heights, IL, US</t>
-        </is>
-      </c>
-      <c r="D123" s="4" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E123" s="4" t="inlineStr">
-        <is>
-          <t>46.0</t>
-        </is>
-      </c>
-      <c r="F123" s="4" t="inlineStr">
-        <is>
-          <t>72.0</t>
-        </is>
-      </c>
-      <c r="G123" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="H123" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="I123" s="4" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="J123" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
-        <is>
-          <t>Incident Response Analyst</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="inlineStr">
-        <is>
-          <t>Alignerr</t>
-        </is>
-      </c>
-      <c r="C124" s="2" t="inlineStr">
-        <is>
-          <t>Dallas, TX</t>
-        </is>
-      </c>
-      <c r="D124" s="2" t="inlineStr"/>
-      <c r="E124" s="2" t="inlineStr"/>
-      <c r="F124" s="2" t="inlineStr"/>
-      <c r="G124" s="2" t="inlineStr"/>
-      <c r="H124" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="I124" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J124" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="4" t="inlineStr">
-        <is>
-          <t>Penetration Tester - TS/SCI with Polygraph</t>
-        </is>
-      </c>
-      <c r="B125" s="4" t="inlineStr">
-        <is>
-          <t>General Dynamics Information Technology</t>
-        </is>
-      </c>
-      <c r="C125" s="4" t="inlineStr">
-        <is>
-          <t>McLean, VA, US</t>
-        </is>
-      </c>
-      <c r="D125" s="4" t="inlineStr"/>
-      <c r="E125" s="4" t="inlineStr">
-        <is>
-          <t>152380.0</t>
-        </is>
-      </c>
-      <c r="F125" s="4" t="inlineStr">
-        <is>
-          <t>206162.0</t>
-        </is>
-      </c>
-      <c r="G125" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="H125" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="I125" s="4" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="J125" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="2" t="inlineStr">
-        <is>
-          <t>Senior Penetration Tester</t>
-        </is>
-      </c>
-      <c r="B126" s="2" t="inlineStr">
-        <is>
-          <t>Quzara LLC</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>Washington, DC, US</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="inlineStr">
-        <is>
-          <t>fulltime</t>
-        </is>
-      </c>
-      <c r="E126" s="2" t="inlineStr"/>
-      <c r="F126" s="2" t="inlineStr"/>
-      <c r="G126" s="2" t="inlineStr"/>
-      <c r="H126" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="I126" s="2" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="J126" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="4" t="inlineStr">
-        <is>
-          <t>Cyber Vulnerability Analyst - Penetration Tester - TS/SCI w/ Poly Required</t>
-        </is>
-      </c>
-      <c r="B127" s="4" t="inlineStr">
-        <is>
-          <t>Parsons</t>
-        </is>
-      </c>
-      <c r="C127" s="4" t="inlineStr">
-        <is>
-          <t>Annapolis Junction, MD, US</t>
-        </is>
-      </c>
-      <c r="D127" s="4" t="inlineStr"/>
-      <c r="E127" s="4" t="inlineStr">
-        <is>
-          <t>134100.0</t>
-        </is>
-      </c>
-      <c r="F127" s="4" t="inlineStr">
-        <is>
-          <t>241400.0</t>
-        </is>
-      </c>
-      <c r="G127" s="4" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="H127" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I127" s="4" t="inlineStr">
-        <is>
-          <t>indeed</t>
-        </is>
-      </c>
-      <c r="J127" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="2" t="inlineStr">
-        <is>
-          <t>AI / Emerging Tech Security Analyst</t>
-        </is>
-      </c>
-      <c r="B128" s="2" t="inlineStr">
-        <is>
-          <t>Alignerr</t>
-        </is>
-      </c>
-      <c r="C128" s="2" t="inlineStr">
-        <is>
-          <t>Boston, MA</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr"/>
-      <c r="E128" s="2" t="inlineStr"/>
-      <c r="F128" s="2" t="inlineStr"/>
-      <c r="G128" s="2" t="inlineStr"/>
-      <c r="H128" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="I128" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J128" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="4" t="inlineStr">
-        <is>
-          <t>Penetration Testing Lead</t>
-        </is>
-      </c>
-      <c r="B129" s="4" t="inlineStr">
-        <is>
-          <t>MANTECH</t>
-        </is>
-      </c>
-      <c r="C129" s="4" t="inlineStr">
-        <is>
-          <t>Chandler, AZ</t>
-        </is>
-      </c>
-      <c r="D129" s="4" t="inlineStr"/>
-      <c r="E129" s="4" t="inlineStr"/>
-      <c r="F129" s="4" t="inlineStr"/>
-      <c r="G129" s="4" t="inlineStr"/>
-      <c r="H129" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="I129" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J129" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="2" t="inlineStr">
-        <is>
-          <t>Penetration Tester - Contract</t>
-        </is>
-      </c>
-      <c r="B130" s="2" t="inlineStr">
-        <is>
-          <t>Bishop Fox</t>
-        </is>
-      </c>
-      <c r="C130" s="2" t="inlineStr"/>
-      <c r="D130" s="2" t="inlineStr"/>
-      <c r="E130" s="2" t="inlineStr"/>
-      <c r="F130" s="2" t="inlineStr"/>
-      <c r="G130" s="2" t="inlineStr"/>
-      <c r="H130" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-19</t>
-        </is>
-      </c>
-      <c r="I130" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J130" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="4" t="inlineStr">
-        <is>
-          <t>Penetration Tester</t>
-        </is>
-      </c>
-      <c r="B131" s="4" t="inlineStr">
-        <is>
-          <t>CyberGuard Advantage</t>
-        </is>
-      </c>
-      <c r="C131" s="4" t="inlineStr"/>
-      <c r="D131" s="4" t="inlineStr"/>
-      <c r="E131" s="4" t="inlineStr"/>
-      <c r="F131" s="4" t="inlineStr"/>
-      <c r="G131" s="4" t="inlineStr"/>
-      <c r="H131" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I131" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J131" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>Security Engineer III (Pen Tester)</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>Deloitte</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>Arlington, VA</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr"/>
-      <c r="E132" s="2" t="inlineStr"/>
-      <c r="F132" s="2" t="inlineStr"/>
-      <c r="G132" s="2" t="inlineStr"/>
-      <c r="H132" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I132" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J132" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="4" t="inlineStr">
-        <is>
-          <t>Senior Application Security Engineer</t>
-        </is>
-      </c>
-      <c r="B133" s="4" t="inlineStr">
-        <is>
-          <t>Insight Global</t>
-        </is>
-      </c>
-      <c r="C133" s="4" t="inlineStr"/>
-      <c r="D133" s="4" t="inlineStr"/>
-      <c r="E133" s="4" t="inlineStr"/>
-      <c r="F133" s="4" t="inlineStr"/>
-      <c r="G133" s="4" t="inlineStr"/>
-      <c r="H133" s="4" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="I133" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J133" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>Red Team Penetration Tester III</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>DirectViz Solutions, LLC</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>Virginia Beach, VA</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr"/>
-      <c r="E134" s="2" t="inlineStr"/>
-      <c r="F134" s="2" t="inlineStr"/>
-      <c r="G134" s="2" t="inlineStr"/>
-      <c r="H134" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J134" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="4" t="inlineStr">
-        <is>
-          <t>Penetration Tester</t>
-        </is>
-      </c>
-      <c r="B135" s="4" t="inlineStr">
-        <is>
-          <t>Akkodis</t>
-        </is>
-      </c>
-      <c r="C135" s="4" t="inlineStr"/>
-      <c r="D135" s="4" t="inlineStr"/>
-      <c r="E135" s="4" t="inlineStr"/>
-      <c r="F135" s="4" t="inlineStr"/>
-      <c r="G135" s="4" t="inlineStr"/>
-      <c r="H135" s="4" t="inlineStr"/>
-      <c r="I135" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J135" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>Senior Penetration Tester</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>Robinhood</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>Bellevue, WA</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr"/>
-      <c r="E136" s="2" t="inlineStr"/>
-      <c r="F136" s="2" t="inlineStr"/>
-      <c r="G136" s="2" t="inlineStr"/>
-      <c r="H136" s="2" t="inlineStr"/>
-      <c r="I136" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J136" s="3" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="4" t="inlineStr">
-        <is>
-          <t>Penetration Tester</t>
-        </is>
-      </c>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t>MANTECH</t>
-        </is>
-      </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>Fort Meade, MD</t>
-        </is>
-      </c>
-      <c r="D137" s="4" t="inlineStr"/>
-      <c r="E137" s="4" t="inlineStr"/>
-      <c r="F137" s="4" t="inlineStr"/>
-      <c r="G137" s="4" t="inlineStr"/>
-      <c r="H137" s="4" t="inlineStr"/>
-      <c r="I137" s="4" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J137" s="5" t="inlineStr">
-        <is>
-          <t>Apply Now</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>Security Engineer</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>Blue Bridge People</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr"/>
-      <c r="D138" s="2" t="inlineStr"/>
-      <c r="E138" s="2" t="inlineStr"/>
-      <c r="F138" s="2" t="inlineStr"/>
-      <c r="G138" s="2" t="inlineStr"/>
-      <c r="H138" s="2" t="inlineStr"/>
-      <c r="I138" s="2" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="J138" s="3" t="inlineStr">
         <is>
           <t>Apply Now</t>
         </is>
@@ -5612,24 +5052,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J118" r:id="rId117"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J119" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J120" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J121" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J122" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J123" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J124" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J125" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J126" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J127" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J128" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J129" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J130" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J131" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J132" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J133" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J134" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J135" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J136" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J137" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J138" r:id="rId137"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>